<commit_message>
feat(H5): Ho tro file Excel mau co dropdown chon Loai bang CN KS THVP CNTT va nut tai file truc tiep tren Admin
</commit_message>
<xml_diff>
--- a/sample_import_khiem.xlsx
+++ b/sample_import_khiem.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DanhSachSinhVien" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,32 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +58,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,220 +452,234 @@
   </sheetPr>
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Mã SV</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Họ Tên</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ngày Sinh</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>GPA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Mã Ngành</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Loại Bằng</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>B210001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Nguyễn Văn An</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>b210001@student.ctuet.edu.vn</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2003-05-15</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>3.65</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>an.b210001@student.ctuet.edu.vn</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2003-01-15</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>7480201</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>KS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>B210002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Trần Thị Bích</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>b210002@student.ctuet.edu.vn</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2003-08-20</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>bich.b210002@student.ctuet.edu.vn</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2003-05-20</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>7480103</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>KS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>B210003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Lê Hoàng Cường</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>b210003@student.ctuet.edu.vn</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2003-12-01</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>cuong.b210003@student.ctuet.edu.vn</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2003-09-12</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>3.1</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>7340101</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>B210004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Phạm Minh Đức</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>b210004@student.ctuet.edu.vn</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2003-03-10</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>duc.b210004@student.ctuet.edu.vn</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2003-11-03</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>7480201</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>THVP</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>B210005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Võ Hoàng Yến</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>b210005@student.ctuet.edu.vn</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2003-07-25</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>yen.b210005@student.ctuet.edu.vn</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2003-07-28</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>7480201</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>CNTT</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Loại bằng không hợp lệ" error="Vui lòng chọn 1 trong các loại văn bằng/chứng chỉ: CN, KS, THVP, CNTT" promptTitle="Chọn Loại Bằng" prompt="Chọn loại văn bằng/chứng chỉ (CN, KS, THVP, CNTT)" type="list">
+      <formula1>"CN,KS,THVP,CNTT"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>